<commit_message>
feat(profesores): implementar gestión de restricciones horarias en el frontend
- Implementa la subida masiva de restricciones desde Excel con validación de errores y advertencia de sobreescritura (upload-restricciones-dialog.tsx).
- Añade columna 'Restricciones' en la tabla de profesores con contador dinámico y acceso a vista rápida (table.tsx, quick-view-restricciones.tsx).
- Integra sistema de pestañas en el modal de edición para separar datos básicos de la gestión de horarios (professor-form-dialog.tsx).
- Crea el componente de gestión individual para añadir y eliminar franjas horarias manualmente (professor-restricciones-tab.tsx).
- Actualiza las interfaces de API y tipos para dar soporte al contador de restricciones (profesores.ts, data.ts).
</commit_message>
<xml_diff>
--- a/docs/Ejemplo restricciones.xlsx
+++ b/docs/Ejemplo restricciones.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TFG\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDD4F75B-0313-4D3B-A172-31A8D78D0CC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDFB817F-803E-408C-BD2A-B055B68521AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31785" yWindow="1800" windowWidth="21600" windowHeight="11385" xr2:uid="{9B37B4F0-CF44-47D5-9DA5-B7C0FB24D9CE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{9B37B4F0-CF44-47D5-9DA5-B7C0FB24D9CE}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
   <si>
     <t>Profesor</t>
   </si>
@@ -47,27 +47,18 @@
     <t>Franja</t>
   </si>
   <si>
-    <t>Juan Pérez Gómez</t>
-  </si>
-  <si>
     <t>L, M</t>
   </si>
   <si>
     <t>08:00-15:00</t>
   </si>
   <si>
-    <t>Ana García</t>
-  </si>
-  <si>
     <t>X , J</t>
   </si>
   <si>
     <t>09:00 - 11:00</t>
   </si>
   <si>
-    <t>Carlos López</t>
-  </si>
-  <si>
     <t>10:00-12:00</t>
   </si>
   <si>
@@ -77,29 +68,41 @@
     <t>15:00-20:00</t>
   </si>
   <si>
-    <t>Elena Martín</t>
-  </si>
-  <si>
     <t>L,M,X,J,V</t>
   </si>
   <si>
     <t>16:00-21:00</t>
   </si>
   <si>
-    <t>david ruiz</t>
-  </si>
-  <si>
     <t>s, d</t>
   </si>
   <si>
     <t>8:00-14:00</t>
+  </si>
+  <si>
+    <t>Adolfo Cobo Garcia</t>
+  </si>
+  <si>
+    <t>Adolfo Garandal Martin</t>
+  </si>
+  <si>
+    <t>Alberto Gonzalez Diez</t>
+  </si>
+  <si>
+    <t>Alberto Martinez Fernandez</t>
+  </si>
+  <si>
+    <t>Alfonso De La Vega Ruiz</t>
+  </si>
+  <si>
+    <t>Alfredo Franco Perez</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -118,6 +121,12 @@
       <sz val="11"/>
       <color rgb="FF1F1F1F"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF09090B"/>
+      <name val="Segoe UI"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -156,7 +165,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
@@ -164,6 +173,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -512,70 +522,70 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="2" t="s">
+    </row>
+    <row r="3" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="2" t="s">
+    </row>
+    <row r="4" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="2" t="s">
+    </row>
+    <row r="5" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="2" t="s">
+    </row>
+    <row r="6" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="2" t="s">
+    </row>
+    <row r="7" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+      <c r="C7" s="2" t="s">
         <v>13</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: actualizar .gitignore y renovar dataset de pruebas
- Ignorados directorios docs/Fichas y docs/Horarios para evitar subir binarios masivos.
- Actualizada plantilla Excel de restricciones de profesores.
- Añadidos documentos de validación (Ficha docente y Horario de prueba) para desarrollo local.
</commit_message>
<xml_diff>
--- a/docs/Ejemplo restricciones.xlsx
+++ b/docs/Ejemplo restricciones.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TFG\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDFB817F-803E-408C-BD2A-B055B68521AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FEE3612-AB65-4037-9885-A89A539893C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{9B37B4F0-CF44-47D5-9DA5-B7C0FB24D9CE}"/>
+    <workbookView xWindow="2985" yWindow="1605" windowWidth="21600" windowHeight="11385" xr2:uid="{9B37B4F0-CF44-47D5-9DA5-B7C0FB24D9CE}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Profesor</t>
   </si>
@@ -53,49 +53,7 @@
     <t>08:00-15:00</t>
   </si>
   <si>
-    <t>X , J</t>
-  </si>
-  <si>
-    <t>09:00 - 11:00</t>
-  </si>
-  <si>
-    <t>10:00-12:00</t>
-  </si>
-  <si>
-    <t>V</t>
-  </si>
-  <si>
-    <t>15:00-20:00</t>
-  </si>
-  <si>
-    <t>L,M,X,J,V</t>
-  </si>
-  <si>
-    <t>16:00-21:00</t>
-  </si>
-  <si>
-    <t>s, d</t>
-  </si>
-  <si>
-    <t>8:00-14:00</t>
-  </si>
-  <si>
-    <t>Adolfo Cobo Garcia</t>
-  </si>
-  <si>
-    <t>Adolfo Garandal Martin</t>
-  </si>
-  <si>
-    <t>Alberto Gonzalez Diez</t>
-  </si>
-  <si>
-    <t>Alberto Martinez Fernandez</t>
-  </si>
-  <si>
-    <t>Alfonso De La Vega Ruiz</t>
-  </si>
-  <si>
-    <t>Alfredo Franco Perez</t>
+    <t>Cristina Tirnauca</t>
   </si>
 </sst>
 </file>
@@ -524,7 +482,7 @@
     </row>
     <row r="2" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>3</v>
@@ -533,60 +491,30 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>13</v>
-      </c>
+    <row r="3" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="3"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+    </row>
+    <row r="4" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="3"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+    </row>
+    <row r="5" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="3"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="3"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+    </row>
+    <row r="7" spans="1:3" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="3"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>